<commit_message>
Refactor app structure and finance module
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,16 +471,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>WM+ DNG</t>
-        </is>
-      </c>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
-        <v>489400</v>
+        <v>80000</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -489,26 +485,26 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Food</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Payment for goods</t>
+          <t>Cầu sân win win, đánh cầu sân lâm gia</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>image</t>
+          <t>text</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>0.95</v>
+        <v>0.8</v>
       </c>
       <c r="J2" t="b">
         <v>0</v>
@@ -517,12 +513,16 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Sân winwin</t>
+        </is>
+      </c>
       <c r="C3" t="n">
-        <v>30000</v>
+        <v>20000</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -559,16 +559,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Phở Thìn</t>
-        </is>
-      </c>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
-        <v>85000</v>
+        <v>30000</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -577,7 +573,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Food</t>
+          <t>Entertainment</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -587,7 +583,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Lunch</t>
+          <t>Đánh cầu lông</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -605,12 +601,16 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Phở Thìn</t>
+        </is>
+      </c>
       <c r="C5" t="n">
-        <v>1630</v>
+        <v>85000</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -619,7 +619,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Food</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -629,16 +629,16 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Hoa ban bap</t>
+          <t>Lunch at Pho Thìn</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>image</t>
+          <t>text</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="J5" t="b">
         <v>0</v>
@@ -647,12 +647,16 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
+          <t>2025-01-15</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Highlands Coffee</t>
+        </is>
+      </c>
       <c r="C6" t="n">
-        <v>20000</v>
+        <v>65000</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -661,17 +665,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Coffee</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Card</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>lấy API</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -680,7 +684,7 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="J6" t="b">
         <v>0</v>
@@ -689,12 +693,16 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
+          <t>2025-01-15</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Test Store</t>
+        </is>
+      </c>
       <c r="C7" t="n">
-        <v>20000</v>
+        <v>50000</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -703,17 +711,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Shopping</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>lấy API của openai</t>
+          <t>Test purchase</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -722,139 +730,9 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="J7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="n">
-        <v>20000</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>VND</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>API AI from OpenAI</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="J8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Petrolimex</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>VND</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Transport</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Bank Transfer</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Đổ xăng chuyển khoản</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="J9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>VND</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Transport</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Bank Transfer</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>đổ xăng chuyển khoản</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="J10" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: use user_id instead of chat_id for data isolation
- Change database schema from chat_id to user_id
- Data now separated by individual user instead of group
- This allows same user to see data across different groups
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,9 +474,13 @@
           <t>2026-05-10</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>quán Tâm</t>
+        </is>
+      </c>
       <c r="C2" t="n">
-        <v>80000</v>
+        <v>200000</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -485,7 +489,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Food</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -495,7 +499,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Cầu sân win win, đánh cầu sân lâm gia</t>
+          <t>Phở</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -504,7 +508,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>0.8</v>
+        <v>0.95</v>
       </c>
       <c r="J2" t="b">
         <v>0</v>
@@ -518,11 +522,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Sân winwin</t>
+          <t>Quán Tâm</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>20000</v>
+        <v>200000</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -531,7 +535,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Entertainment</t>
+          <t>Food</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -541,7 +545,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Đánh cầu lông</t>
+          <t>Phở</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -564,7 +568,7 @@
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
-        <v>30000</v>
+        <v>200000</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -573,7 +577,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Entertainment</t>
+          <t>Food</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -583,7 +587,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Đánh cầu lông</t>
+          <t>Phở</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -595,144 +599,6 @@
         <v>0.95</v>
       </c>
       <c r="J4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Phở Thìn</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>85000</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>VND</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Food</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Lunch at Pho Thìn</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="J5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2025-01-15</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Highlands Coffee</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>65000</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>VND</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Coffee</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Card</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2025-01-15</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Test Store</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>50000</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>VND</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Shopping</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Cash</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Test purchase</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: update i18n multi lanaguge
</commit_message>
<xml_diff>
--- a/data/expenses.xlsx
+++ b/data/expenses.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,13 +474,9 @@
           <t>2026-05-10</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>quán Tâm</t>
-        </is>
-      </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
-        <v>200000</v>
+        <v>30000</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -489,7 +485,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Food</t>
+          <t>Income</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -499,7 +495,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Phở</t>
+          <t>salary from company</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -508,7 +504,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="J2" t="b">
         <v>0</v>
@@ -522,11 +518,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Quán Tâm</t>
+          <t>quán gần chung cư</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>200000</v>
+        <v>30000</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -545,7 +541,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Phở</t>
+          <t>ăn bún chả hà nội</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -557,48 +553,6 @@
         <v>0.95</v>
       </c>
       <c r="J3" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="n">
-        <v>200000</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>VND</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Food</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Phở</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="I4" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="J4" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>